<commit_message>
tracker: mark REV-001 done -- Sprint 9/ML9 1 of 2 stories complete
REV-001 flipped to Done, propagated through Epic ML9-EP01 (1/2
stories -- In Progress, REV-002 remaining), Milestone ML9 (1/2 --
In Progress), Sprint SP09 (1/2 -- In Progress), Phase Tracker PH2,
and the Dashboard.

Dashboard: Overall Progress 0.568 (was 0.542), Completed Stories 36
(was 35). Completed Milestones/Epics unchanged (ML9-EP01/ML9 not yet
complete). Current Milestone/Sprint remain ML9/SP09.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.542</v>
+        <v>0.568</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.542</v>
+        <v>0.568</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5917,11 +5917,11 @@
       <c r="I10" s="12"/>
       <c r="J10" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B10)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B10),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K10" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B10,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J10=1,"✅ Completed",IF(J10&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="L10" s="12" t="n">
         <v>0</v>
@@ -6865,11 +6865,11 @@
       <c r="I16" s="10"/>
       <c r="J16" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C16)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C16),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K16" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C16,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J16=1,"✅ Completed",IF(J16&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8035,15 +8035,15 @@
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A10)*(Stories!$P$2:$P$200))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="11" t="n">
         <f aca="false">IFERROR(H10/G10,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J10" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A10,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I10=1,"✅ Completed",IF(I10&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>87</v>
@@ -10441,7 +10441,7 @@
       <c r="K36" s="10"/>
       <c r="L36" s="10"/>
       <c r="M36" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N36" s="10"/>
       <c r="O36" s="10" t="s">

</xml_diff>

<commit_message>
chore(tracker): sync REV-002 completion through Milestone ML9
Story REV-002 marked Done, propagated up the rollup hierarchy:
- Epic ML9-EP01: In Progress -> Completed (both its stories, REV-001
  and REV-002, are now Done)
- Milestone ML9: In Progress -> Completed
- Sprint SP09: In Progress -> Completed (2/2 stories done)
- Phase PH2 progress: 0.72 -> 0.76 (13/25 -> 14/25... average across
  PH2's stories)
- Dashboard: Overall Progress 0.568 -> 0.594, Completed Milestones
  8 -> 9, Completed Epics 15 -> 16, Completed Stories 36 -> 37

Applied via direct XML cell patch (unzip/patch/rezip) to preserve the
workbook's existing formatting; each of the 14 changed cells verified
individually against the expected recomputation before replacing the
real file, and diff-checked to confirm no other cell was touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.568</v>
+        <v>0.594</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4525,7 +4525,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.72</v>
+        <v>0.76</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5917,11 +5917,11 @@
       <c r="I10" s="12"/>
       <c r="J10" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B10)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B10),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K10" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B10,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J10=1,"✅ Completed",IF(J10&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L10" s="12" t="n">
         <v>0</v>
@@ -6865,11 +6865,11 @@
       <c r="I16" s="10"/>
       <c r="J16" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C16)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C16),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K16" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C16,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J16=1,"✅ Completed",IF(J16&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8035,15 +8035,15 @@
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A10)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10" s="11" t="n">
         <f aca="false">IFERROR(H10/G10,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J10" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A10,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I10=1,"✅ Completed",IF(I10&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>87</v>
@@ -10484,7 +10484,7 @@
       <c r="K37" s="10"/>
       <c r="L37" s="10"/>
       <c r="M37" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N37" s="10"/>
       <c r="O37" s="10" t="s">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="P37" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M37)),1,IF(ISNUMBER(SEARCH("In Progress",M37)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="66" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore(tracker): sync LEAD-001 completion (Sprint 10 1 of 2)
Story LEAD-001 marked Done, propagated up the rollup hierarchy:
- Epic ML10-EP01: Planned -> In Progress (0.5, 1/2 stories done)
- Milestone ML10: Planned -> In Progress (0.5)
- Sprint SP10: Planned -> In Progress (1/2 stories done)
- Phase PH2 progress: 0.76 -> 0.8
- Dashboard: Overall Progress 0.594 -> 0.62, Completed Stories 37 -> 38
  (Completed Milestones/Epics unchanged at 9/16 - neither ML10 nor
  ML10-EP01 is fully complete yet, LEAD-002 remains)

Applied via direct XML cell patch (unzip/patch/rezip), each of the 12
changed cells verified individually before replacing the real file,
and diff-checked to confirm no other cell was touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.594</v>
+        <v>0.62</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5949,11 +5949,11 @@
       <c r="I11" s="12"/>
       <c r="J11" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B11)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B11),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K11" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B11,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J11=1,"✅ Completed",IF(J11&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="L11" s="12" t="n">
         <v>0</v>
@@ -6894,11 +6894,11 @@
       <c r="I17" s="10"/>
       <c r="J17" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C17)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C17),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K17" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C17,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J17=1,"✅ Completed",IF(J17&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8074,15 +8074,15 @@
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A11)*(Stories!$P$2:$P$200))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" s="11" t="n">
         <f aca="false">IFERROR(H11/G11,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J11" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A11,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I11=1,"✅ Completed",IF(I11&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>90</v>
@@ -10527,7 +10527,7 @@
       <c r="K38" s="10"/>
       <c r="L38" s="10"/>
       <c r="M38" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N38" s="10"/>
       <c r="O38" s="10" t="s">
@@ -10535,7 +10535,7 @@
       </c>
       <c r="P38" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M38)),1,IF(ISNUMBER(SEARCH("In Progress",M38)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="52.5" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore(tracker): fix stale Dashboard chart-data story-status counts
The Dashboard's "Chart Data — Story Status" mini-table (used to feed a
chart visual, distinct from the correctly-synced "Completed Stories"
metric) had gone stale independently of the per-story tracker sync
process - it showed Done=28/Not Started=18 (summing to 46, not 47)
against the real, current counts of Done=38/Not Started=9 (summing to
47, matching Total Stories). This table is a plain hardcoded snapshot,
not a formula, so it was never automatically kept in sync and had
drifted unnoticed across several stories' worth of closeouts.

Verified via a structural diff against the pre-fix file that only
these two cells (J7, J10) changed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4421,7 +4421,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4493,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore(tracker): sync LEAD-002 completion - Sprint 10 and ML10 done
Story LEAD-002 marked Done, propagated up the rollup hierarchy:
- Epic ML10-EP01: In Progress -> Completed (2/2 stories done)
- Milestone ML10: In Progress -> Completed
- Sprint SP10: In Progress -> Completed (2/2 stories done)
- Phase PH2 progress: 0.8 -> 0.84
- Dashboard: Overall Progress 0.62 -> 0.646, Completed Milestones
  9 -> 10, Completed Epics 16 -> 17, Completed Stories 38 -> 39;
  also corrected the "Chart Data - Story Status" mini-table's Done/Not
  Started split to 39/8 (still summing to 47)

Applied via direct XML cell patch (unzip/patch/rezip), each of the 16
changed cells verified individually before replacing the real file,
and diff-checked to confirm no other cell was touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.62</v>
+        <v>0.646</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4421,7 +4421,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4493,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4525,7 +4525,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5949,11 +5949,11 @@
       <c r="I11" s="12"/>
       <c r="J11" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B11)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B11),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K11" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B11,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J11=1,"✅ Completed",IF(J11&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L11" s="12" t="n">
         <v>0</v>
@@ -6894,11 +6894,11 @@
       <c r="I17" s="10"/>
       <c r="J17" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C17)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C17),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K17" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C17,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J17=1,"✅ Completed",IF(J17&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8074,15 +8074,15 @@
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A11)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I11" s="11" t="n">
         <f aca="false">IFERROR(H11/G11,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J11" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A11,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I11=1,"✅ Completed",IF(I11&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>90</v>
@@ -10570,7 +10570,7 @@
       <c r="K39" s="10"/>
       <c r="L39" s="10"/>
       <c r="M39" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N39" s="10"/>
       <c r="O39" s="10" t="s">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="P39" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M39)),1,IF(ISNUMBER(SEARCH("In Progress",M39)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="78.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore(tracker): sync ADM-001 completion (Sprint 11 1 of 2)
Story ADM-001 marked Done, propagated up the rollup hierarchy:
- Epic ML11-EP01: Planned -> In Progress (0.5, 1/2 stories done)
- Milestone ML11: Planned -> In Progress (0.5)
- Sprint SP11: Planned -> In Progress (1/2 stories done)
- Phase PH2 progress: 0.84 -> 0.88
- Dashboard: Overall Progress 0.646 -> 0.672, Completed Stories
  39 -> 40 (Completed Milestones/Epics unchanged at 10/17 - neither
  ML11 nor ML11-EP01 is fully complete yet, ADM-002 remains); Chart
  Data Done/Not Started split updated to 40/7 (still summing to 47)

Applied via direct XML cell patch (unzip/patch/rezip), each of the 14
changed cells verified individually before replacing the real file,
and diff-checked to confirm no other cell was touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.646</v>
+        <v>0.672</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4421,7 +4421,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4493,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5981,11 +5981,11 @@
       <c r="I12" s="12"/>
       <c r="J12" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B12)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B12),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K12" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B12,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J12=1,"✅ Completed",IF(J12&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="L12" s="12" t="n">
         <v>0</v>
@@ -6923,11 +6923,11 @@
       <c r="I18" s="10"/>
       <c r="J18" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C18)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C18),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K18" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C18,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J18=1,"✅ Completed",IF(J18&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8113,15 +8113,15 @@
       </c>
       <c r="H12" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A12)*(Stories!$P$2:$P$200))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" s="11" t="n">
         <f aca="false">IFERROR(H12/G12,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J12" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A12,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I12=1,"✅ Completed",IF(I12&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>93</v>
@@ -10613,7 +10613,7 @@
       <c r="K40" s="10"/>
       <c r="L40" s="10"/>
       <c r="M40" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N40" s="10"/>
       <c r="O40" s="10" t="s">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="P40" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M40)),1,IF(ISNUMBER(SEARCH("In Progress",M40)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="66" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore(tracker): sync ADM-002 completion - Sprint 11 and ML11 complete
Story ADM-002 marked Done, propagated up the rollup hierarchy:
- Epic ML11-EP01: In Progress -> Completed (2/2 stories done)
- Milestone ML11: In Progress -> Completed
- Sprint SP11: In Progress -> Completed (2/2 stories done)
- Phase PH2 progress: 0.88 -> 0.92
- Dashboard: Overall Progress 0.672 -> 0.698, Completed Milestones
  10 -> 11, Completed Epics 17 -> 18, Completed Stories 40 -> 41;
  Chart Data Done/Not Started split updated to 41/6 (still summing
  to 47)

Applied via direct XML cell patch (unzip/patch/rezip), each of the 16
changed cells verified individually before replacing the real file,
and diff-checked to confirm no other cell was touched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.672</v>
+        <v>0.698</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4421,7 +4421,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4493,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4525,7 +4525,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5981,11 +5981,11 @@
       <c r="I12" s="12"/>
       <c r="J12" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B12)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B12),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K12" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B12,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J12=1,"✅ Completed",IF(J12&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L12" s="12" t="n">
         <v>0</v>
@@ -6923,11 +6923,11 @@
       <c r="I18" s="10"/>
       <c r="J18" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C18)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C18),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K18" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C18,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J18=1,"✅ Completed",IF(J18&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8113,15 +8113,15 @@
       </c>
       <c r="H12" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A12)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I12" s="11" t="n">
         <f aca="false">IFERROR(H12/G12,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J12" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A12,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I12=1,"✅ Completed",IF(I12&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>93</v>
@@ -10656,7 +10656,7 @@
       <c r="K41" s="10"/>
       <c r="L41" s="10"/>
       <c r="M41" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N41" s="10"/>
       <c r="O41" s="10" t="s">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="P41" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M41)),1,IF(ISNUMBER(SEARCH("In Progress",M41)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="78.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>